<commit_message>
hit hissiyatı ve combat polish
</commit_message>
<xml_diff>
--- a/Exponentia Mobs/exponentia_secili_mob_boss_havuzu.xlsx
+++ b/Exponentia Mobs/exponentia_secili_mob_boss_havuzu.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tunag\OneDrive\Masaüstü\exponentia mobs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROJECTS\YMH212-Exponentia\Exponentia Mobs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EEBBEDA-A337-4AB4-9CC7-03B72D8C5DFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A40F7AD3-C024-4924-B2CE-4DFACB1A61CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Basic Moblar" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="168">
   <si>
     <t>Basic Moblar</t>
   </si>
@@ -308,18 +308,6 @@
     <t>Düşen kor mermileri + ritmik darbe</t>
   </si>
   <si>
-    <t>Pythia’nın Gölgesi</t>
-  </si>
-  <si>
-    <t>Mor dumanlardan dev kadın silueti</t>
-  </si>
-  <si>
-    <t>Kavisli S-şeklinde mermiler atar; ekranı negatif renge çevirir</t>
-  </si>
-  <si>
-    <t>Kavisli patternler + görsel bozulma</t>
-  </si>
-  <si>
     <t>Aetos Dios</t>
   </si>
   <si>
@@ -330,24 +318,6 @@
   </si>
   <si>
     <t>İtme rüzgarı + gölge telegraph + halka dalga</t>
-  </si>
-  <si>
-    <t>Ares’in Kuşatma Kulesi</t>
-  </si>
-  <si>
-    <t>Canlı bir kuşatma kulesi</t>
-  </si>
-  <si>
-    <t>Pencerelerden mermi yağar; parçalanınca berserk komutan çıkar</t>
-  </si>
-  <si>
-    <t>Çoklu mermi pencereleri + ikinci faz komutan</t>
-  </si>
-  <si>
-    <t>Aşırı Yüksek</t>
-  </si>
-  <si>
-    <t>Düşük/Orta</t>
   </si>
   <si>
     <t>Kronos, Zamanın Efendisi</t>
@@ -1033,19 +1003,19 @@
     </row>
     <row r="5" spans="1:10" ht="42.65" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>18</v>
@@ -1054,7 +1024,7 @@
         <v>18</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>19</v>
@@ -1062,7 +1032,7 @@
     </row>
     <row r="6" spans="1:10" ht="42.65" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>20</v>
@@ -1074,7 +1044,7 @@
         <v>22</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>18</v>
@@ -1091,7 +1061,7 @@
     </row>
     <row r="7" spans="1:10" ht="42.65" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>24</v>
@@ -1100,10 +1070,10 @@
         <v>25</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>26</v>
@@ -1120,7 +1090,7 @@
     </row>
     <row r="8" spans="1:10" ht="42.65" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>28</v>
@@ -1149,7 +1119,7 @@
     </row>
     <row r="9" spans="1:10" ht="42.65" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>33</v>
@@ -1178,7 +1148,7 @@
     </row>
     <row r="10" spans="1:10" ht="42.65" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>39</v>
@@ -1207,7 +1177,7 @@
     </row>
     <row r="11" spans="1:10" ht="42.65" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>43</v>
@@ -1236,7 +1206,7 @@
     </row>
     <row r="12" spans="1:10" ht="42.65" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>48</v>
@@ -1245,10 +1215,10 @@
         <v>49</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>26</v>
@@ -1265,7 +1235,7 @@
     </row>
     <row r="13" spans="1:10" ht="42.65" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>51</v>
@@ -1294,13 +1264,13 @@
     </row>
     <row r="14" spans="1:10" ht="42.65" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>55</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>56</v>
@@ -1323,7 +1293,7 @@
     </row>
     <row r="15" spans="1:10" ht="42.65" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>58</v>
@@ -1332,10 +1302,10 @@
         <v>59</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>37</v>
@@ -1352,31 +1322,31 @@
     </row>
     <row r="16" spans="1:10" ht="42.65" customHeight="1">
       <c r="A16" s="7" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="B16" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E16" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="F16" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>151</v>
-      </c>
       <c r="G16" s="7" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" ht="42.65" customHeight="1"/>
@@ -1460,7 +1430,7 @@
     </row>
     <row r="5" spans="1:8" ht="42.65" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>61</v>
@@ -1472,7 +1442,7 @@
         <v>63</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>26</v>
@@ -1486,25 +1456,25 @@
     </row>
     <row r="6" spans="1:8" ht="73.5" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>50</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>47</v>
@@ -1512,7 +1482,7 @@
     </row>
     <row r="7" spans="1:8" ht="42.65" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>65</v>
@@ -1524,13 +1494,13 @@
         <v>67</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>47</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>26</v>
@@ -1538,7 +1508,7 @@
     </row>
     <row r="8" spans="1:8" ht="42.65" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>68</v>
@@ -1547,13 +1517,13 @@
         <v>69</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>32</v>
@@ -1564,7 +1534,7 @@
     </row>
     <row r="9" spans="1:8" ht="42.65" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>70</v>
@@ -1661,16 +1631,16 @@
     </row>
     <row r="5" spans="1:7" ht="42.65" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>75</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>47</v>
@@ -1684,7 +1654,7 @@
     </row>
     <row r="6" spans="1:7" ht="42.65" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>76</v>
@@ -1693,7 +1663,7 @@
         <v>77</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>23</v>
@@ -1707,16 +1677,16 @@
     </row>
     <row r="7" spans="1:7" ht="42.65" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>78</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>47</v>
@@ -1885,7 +1855,7 @@
         <v>47</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>47</v>
@@ -1905,427 +1875,399 @@
         <v>97</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>47</v>
+        <v>98</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>47</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="42.65" customHeight="1">
       <c r="A10" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>102</v>
-      </c>
       <c r="F10" s="1" t="s">
-        <v>103</v>
+        <v>23</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>47</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="42.65" customHeight="1">
       <c r="A11" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>107</v>
-      </c>
       <c r="E11" s="1" t="s">
-        <v>108</v>
+        <v>47</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>108</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="42.65" customHeight="1">
       <c r="A12" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="E12" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="42.65" customHeight="1">
+      <c r="A13" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="B13" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="42.65" customHeight="1">
-      <c r="A13" s="4" t="s">
+      <c r="C13" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="D13" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="F13" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="G13" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="G13" s="1" t="s">
-        <v>47</v>
-      </c>
     </row>
     <row r="14" spans="1:7" ht="42.65" customHeight="1">
-      <c r="A14" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>47</v>
-      </c>
+      <c r="A14" s="4"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
     </row>
     <row r="15" spans="1:7" ht="42.65" customHeight="1">
-      <c r="A15" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>47</v>
-      </c>
+      <c r="A15" s="4"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="26" spans="1:7">
       <c r="A26" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>